<commit_message>
Add Article 3 experimental data
</commit_message>
<xml_diff>
--- a/data/processed/clean_article_data.xlsx
+++ b/data/processed/clean_article_data.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
-  <workbookPr defaultThemeVersion="202300"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\moham\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\AI\ai-corrosion-roadmap\ai_corrosion_quince\data\processed\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{4A59EF27-E088-451A-8722-15DCFEF932A0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{35E0F9D8-A982-48AD-A5F0-0FE6508BA49A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1330" yWindow="1360" windowWidth="19200" windowHeight="11170" xr2:uid="{CAB2D7DB-2A5C-44DE-8AD5-94CA0C6BC49C}"/>
+    <workbookView xWindow="990" yWindow="1020" windowWidth="19200" windowHeight="11170" xr2:uid="{CAB2D7DB-2A5C-44DE-8AD5-94CA0C6BC49C}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="358" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="474" uniqueCount="43">
   <si>
     <t>row_id</t>
   </si>
@@ -150,6 +150,24 @@
   </si>
   <si>
     <t>max EIS IE at 328 K</t>
+  </si>
+  <si>
+    <t>P3</t>
+  </si>
+  <si>
+    <t>H2SO4</t>
+  </si>
+  <si>
+    <t>P3_Table2</t>
+  </si>
+  <si>
+    <t>max polarization IE in P3</t>
+  </si>
+  <si>
+    <t>P3_Table3</t>
+  </si>
+  <si>
+    <t>max EIS IE in P3</t>
   </si>
 </sst>
 </file>
@@ -521,7 +539,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A6D92F60-C5DD-497B-B69E-54DA44CF4FAF}">
-  <dimension ref="A1:P42"/>
+  <dimension ref="A1:P56"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
     <row r="1" spans="1:16" x14ac:dyDescent="0.35">
@@ -2543,6 +2561,676 @@
         <v>36</v>
       </c>
     </row>
+    <row r="43" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="A43">
+        <v>45</v>
+      </c>
+      <c r="B43" t="s">
+        <v>37</v>
+      </c>
+      <c r="C43">
+        <v>2023</v>
+      </c>
+      <c r="D43" t="s">
+        <v>17</v>
+      </c>
+      <c r="E43" t="s">
+        <v>18</v>
+      </c>
+      <c r="F43" t="s">
+        <v>38</v>
+      </c>
+      <c r="G43">
+        <v>1</v>
+      </c>
+      <c r="H43">
+        <v>298</v>
+      </c>
+      <c r="I43">
+        <v>30</v>
+      </c>
+      <c r="J43">
+        <v>0</v>
+      </c>
+      <c r="K43" t="s">
+        <v>20</v>
+      </c>
+      <c r="L43">
+        <v>0</v>
+      </c>
+      <c r="M43" t="s">
+        <v>21</v>
+      </c>
+      <c r="N43" t="s">
+        <v>22</v>
+      </c>
+      <c r="O43" t="s">
+        <v>39</v>
+      </c>
+      <c r="P43" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="44" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="A44">
+        <v>46</v>
+      </c>
+      <c r="B44" t="s">
+        <v>37</v>
+      </c>
+      <c r="C44">
+        <v>2023</v>
+      </c>
+      <c r="D44" t="s">
+        <v>17</v>
+      </c>
+      <c r="E44" t="s">
+        <v>18</v>
+      </c>
+      <c r="F44" t="s">
+        <v>38</v>
+      </c>
+      <c r="G44">
+        <v>1</v>
+      </c>
+      <c r="H44">
+        <v>298</v>
+      </c>
+      <c r="I44">
+        <v>30</v>
+      </c>
+      <c r="J44">
+        <v>200</v>
+      </c>
+      <c r="K44" t="s">
+        <v>20</v>
+      </c>
+      <c r="L44">
+        <v>51.5</v>
+      </c>
+      <c r="M44" t="s">
+        <v>25</v>
+      </c>
+      <c r="N44" t="s">
+        <v>22</v>
+      </c>
+      <c r="O44" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="45" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="A45">
+        <v>47</v>
+      </c>
+      <c r="B45" t="s">
+        <v>37</v>
+      </c>
+      <c r="C45">
+        <v>2023</v>
+      </c>
+      <c r="D45" t="s">
+        <v>17</v>
+      </c>
+      <c r="E45" t="s">
+        <v>18</v>
+      </c>
+      <c r="F45" t="s">
+        <v>38</v>
+      </c>
+      <c r="G45">
+        <v>1</v>
+      </c>
+      <c r="H45">
+        <v>298</v>
+      </c>
+      <c r="I45">
+        <v>30</v>
+      </c>
+      <c r="J45">
+        <v>400</v>
+      </c>
+      <c r="K45" t="s">
+        <v>20</v>
+      </c>
+      <c r="L45">
+        <v>73.3</v>
+      </c>
+      <c r="M45" t="s">
+        <v>25</v>
+      </c>
+      <c r="N45" t="s">
+        <v>22</v>
+      </c>
+      <c r="O45" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="46" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="A46">
+        <v>48</v>
+      </c>
+      <c r="B46" t="s">
+        <v>37</v>
+      </c>
+      <c r="C46">
+        <v>2023</v>
+      </c>
+      <c r="D46" t="s">
+        <v>17</v>
+      </c>
+      <c r="E46" t="s">
+        <v>18</v>
+      </c>
+      <c r="F46" t="s">
+        <v>38</v>
+      </c>
+      <c r="G46">
+        <v>1</v>
+      </c>
+      <c r="H46">
+        <v>298</v>
+      </c>
+      <c r="I46">
+        <v>30</v>
+      </c>
+      <c r="J46">
+        <v>600</v>
+      </c>
+      <c r="K46" t="s">
+        <v>20</v>
+      </c>
+      <c r="L46">
+        <v>78.900000000000006</v>
+      </c>
+      <c r="M46" t="s">
+        <v>25</v>
+      </c>
+      <c r="N46" t="s">
+        <v>22</v>
+      </c>
+      <c r="O46" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="47" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="A47">
+        <v>49</v>
+      </c>
+      <c r="B47" t="s">
+        <v>37</v>
+      </c>
+      <c r="C47">
+        <v>2023</v>
+      </c>
+      <c r="D47" t="s">
+        <v>17</v>
+      </c>
+      <c r="E47" t="s">
+        <v>18</v>
+      </c>
+      <c r="F47" t="s">
+        <v>38</v>
+      </c>
+      <c r="G47">
+        <v>1</v>
+      </c>
+      <c r="H47">
+        <v>298</v>
+      </c>
+      <c r="I47">
+        <v>30</v>
+      </c>
+      <c r="J47">
+        <v>800</v>
+      </c>
+      <c r="K47" t="s">
+        <v>20</v>
+      </c>
+      <c r="L47">
+        <v>84</v>
+      </c>
+      <c r="M47" t="s">
+        <v>25</v>
+      </c>
+      <c r="N47" t="s">
+        <v>22</v>
+      </c>
+      <c r="O47" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="48" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="A48">
+        <v>50</v>
+      </c>
+      <c r="B48" t="s">
+        <v>37</v>
+      </c>
+      <c r="C48">
+        <v>2023</v>
+      </c>
+      <c r="D48" t="s">
+        <v>17</v>
+      </c>
+      <c r="E48" t="s">
+        <v>18</v>
+      </c>
+      <c r="F48" t="s">
+        <v>38</v>
+      </c>
+      <c r="G48">
+        <v>1</v>
+      </c>
+      <c r="H48">
+        <v>298</v>
+      </c>
+      <c r="I48">
+        <v>30</v>
+      </c>
+      <c r="J48">
+        <v>1000</v>
+      </c>
+      <c r="K48" t="s">
+        <v>20</v>
+      </c>
+      <c r="L48">
+        <v>86.3</v>
+      </c>
+      <c r="M48" t="s">
+        <v>25</v>
+      </c>
+      <c r="N48" t="s">
+        <v>22</v>
+      </c>
+      <c r="O48" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="49" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="A49">
+        <v>51</v>
+      </c>
+      <c r="B49" t="s">
+        <v>37</v>
+      </c>
+      <c r="C49">
+        <v>2023</v>
+      </c>
+      <c r="D49" t="s">
+        <v>17</v>
+      </c>
+      <c r="E49" t="s">
+        <v>18</v>
+      </c>
+      <c r="F49" t="s">
+        <v>38</v>
+      </c>
+      <c r="G49">
+        <v>1</v>
+      </c>
+      <c r="H49">
+        <v>298</v>
+      </c>
+      <c r="I49">
+        <v>30</v>
+      </c>
+      <c r="J49">
+        <v>1200</v>
+      </c>
+      <c r="K49" t="s">
+        <v>20</v>
+      </c>
+      <c r="L49">
+        <v>94.5</v>
+      </c>
+      <c r="M49" t="s">
+        <v>25</v>
+      </c>
+      <c r="N49" t="s">
+        <v>22</v>
+      </c>
+      <c r="O49" t="s">
+        <v>39</v>
+      </c>
+      <c r="P49" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="50" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="A50">
+        <v>52</v>
+      </c>
+      <c r="B50" t="s">
+        <v>37</v>
+      </c>
+      <c r="C50">
+        <v>2023</v>
+      </c>
+      <c r="D50" t="s">
+        <v>17</v>
+      </c>
+      <c r="E50" t="s">
+        <v>18</v>
+      </c>
+      <c r="F50" t="s">
+        <v>38</v>
+      </c>
+      <c r="G50">
+        <v>1</v>
+      </c>
+      <c r="H50">
+        <v>298</v>
+      </c>
+      <c r="I50">
+        <v>30</v>
+      </c>
+      <c r="J50">
+        <v>0</v>
+      </c>
+      <c r="K50" t="s">
+        <v>27</v>
+      </c>
+      <c r="L50">
+        <v>0</v>
+      </c>
+      <c r="M50" t="s">
+        <v>21</v>
+      </c>
+      <c r="N50" t="s">
+        <v>22</v>
+      </c>
+      <c r="O50" t="s">
+        <v>41</v>
+      </c>
+      <c r="P50" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="51" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="A51">
+        <v>53</v>
+      </c>
+      <c r="B51" t="s">
+        <v>37</v>
+      </c>
+      <c r="C51">
+        <v>2023</v>
+      </c>
+      <c r="D51" t="s">
+        <v>17</v>
+      </c>
+      <c r="E51" t="s">
+        <v>18</v>
+      </c>
+      <c r="F51" t="s">
+        <v>38</v>
+      </c>
+      <c r="G51">
+        <v>1</v>
+      </c>
+      <c r="H51">
+        <v>298</v>
+      </c>
+      <c r="I51">
+        <v>30</v>
+      </c>
+      <c r="J51">
+        <v>200</v>
+      </c>
+      <c r="K51" t="s">
+        <v>27</v>
+      </c>
+      <c r="L51">
+        <v>58.2</v>
+      </c>
+      <c r="M51" t="s">
+        <v>25</v>
+      </c>
+      <c r="N51" t="s">
+        <v>22</v>
+      </c>
+      <c r="O51" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="52" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="A52">
+        <v>54</v>
+      </c>
+      <c r="B52" t="s">
+        <v>37</v>
+      </c>
+      <c r="C52">
+        <v>2023</v>
+      </c>
+      <c r="D52" t="s">
+        <v>17</v>
+      </c>
+      <c r="E52" t="s">
+        <v>18</v>
+      </c>
+      <c r="F52" t="s">
+        <v>38</v>
+      </c>
+      <c r="G52">
+        <v>1</v>
+      </c>
+      <c r="H52">
+        <v>298</v>
+      </c>
+      <c r="I52">
+        <v>30</v>
+      </c>
+      <c r="J52">
+        <v>400</v>
+      </c>
+      <c r="K52" t="s">
+        <v>27</v>
+      </c>
+      <c r="L52">
+        <v>74.5</v>
+      </c>
+      <c r="M52" t="s">
+        <v>25</v>
+      </c>
+      <c r="N52" t="s">
+        <v>22</v>
+      </c>
+      <c r="O52" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="53" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="A53">
+        <v>55</v>
+      </c>
+      <c r="B53" t="s">
+        <v>37</v>
+      </c>
+      <c r="C53">
+        <v>2023</v>
+      </c>
+      <c r="D53" t="s">
+        <v>17</v>
+      </c>
+      <c r="E53" t="s">
+        <v>18</v>
+      </c>
+      <c r="F53" t="s">
+        <v>38</v>
+      </c>
+      <c r="G53">
+        <v>1</v>
+      </c>
+      <c r="H53">
+        <v>298</v>
+      </c>
+      <c r="I53">
+        <v>30</v>
+      </c>
+      <c r="J53">
+        <v>600</v>
+      </c>
+      <c r="K53" t="s">
+        <v>27</v>
+      </c>
+      <c r="L53">
+        <v>76.3</v>
+      </c>
+      <c r="M53" t="s">
+        <v>25</v>
+      </c>
+      <c r="N53" t="s">
+        <v>22</v>
+      </c>
+      <c r="O53" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="54" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="A54">
+        <v>56</v>
+      </c>
+      <c r="B54" t="s">
+        <v>37</v>
+      </c>
+      <c r="C54">
+        <v>2023</v>
+      </c>
+      <c r="D54" t="s">
+        <v>17</v>
+      </c>
+      <c r="E54" t="s">
+        <v>18</v>
+      </c>
+      <c r="F54" t="s">
+        <v>38</v>
+      </c>
+      <c r="G54">
+        <v>1</v>
+      </c>
+      <c r="H54">
+        <v>298</v>
+      </c>
+      <c r="I54">
+        <v>30</v>
+      </c>
+      <c r="J54">
+        <v>800</v>
+      </c>
+      <c r="K54" t="s">
+        <v>27</v>
+      </c>
+      <c r="L54">
+        <v>79.900000000000006</v>
+      </c>
+      <c r="M54" t="s">
+        <v>25</v>
+      </c>
+      <c r="N54" t="s">
+        <v>22</v>
+      </c>
+      <c r="O54" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="55" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="A55">
+        <v>57</v>
+      </c>
+      <c r="B55" t="s">
+        <v>37</v>
+      </c>
+      <c r="C55">
+        <v>2023</v>
+      </c>
+      <c r="D55" t="s">
+        <v>17</v>
+      </c>
+      <c r="E55" t="s">
+        <v>18</v>
+      </c>
+      <c r="F55" t="s">
+        <v>38</v>
+      </c>
+      <c r="G55">
+        <v>1</v>
+      </c>
+      <c r="H55">
+        <v>298</v>
+      </c>
+      <c r="I55">
+        <v>30</v>
+      </c>
+      <c r="J55">
+        <v>1000</v>
+      </c>
+      <c r="K55" t="s">
+        <v>27</v>
+      </c>
+      <c r="L55">
+        <v>82.9</v>
+      </c>
+      <c r="M55" t="s">
+        <v>25</v>
+      </c>
+      <c r="N55" t="s">
+        <v>22</v>
+      </c>
+      <c r="O55" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="56" spans="1:16" x14ac:dyDescent="0.35">
+      <c r="A56">
+        <v>58</v>
+      </c>
+      <c r="B56" t="s">
+        <v>37</v>
+      </c>
+      <c r="C56">
+        <v>2023</v>
+      </c>
+      <c r="D56" t="s">
+        <v>17</v>
+      </c>
+      <c r="E56" t="s">
+        <v>18</v>
+      </c>
+      <c r="F56" t="s">
+        <v>38</v>
+      </c>
+      <c r="G56">
+        <v>1</v>
+      </c>
+      <c r="H56">
+        <v>298</v>
+      </c>
+      <c r="I56">
+        <v>30</v>
+      </c>
+      <c r="J56">
+        <v>1200</v>
+      </c>
+      <c r="K56" t="s">
+        <v>27</v>
+      </c>
+      <c r="L56">
+        <v>90.7</v>
+      </c>
+      <c r="M56" t="s">
+        <v>25</v>
+      </c>
+      <c r="N56" t="s">
+        <v>22</v>
+      </c>
+      <c r="O56" t="s">
+        <v>41</v>
+      </c>
+      <c r="P56" t="s">
+        <v>42</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>